<commit_message>
seo-log: actualizar bitacora con hallazgos y acciones del 11/07
- optimizacion de imagenes de producto (ver commit 4d732d2)
- nota: auditoria sin Claude en Chrome disponible
- estado del proyecto Mundialista: sin cambios, partido aun no jugado
- propuesta pendiente: reducir friccion en formulario de descuento
</commit_message>
<xml_diff>
--- a/seo-log/vitacora de SEO PP.xlsx
+++ b/seo-log/vitacora de SEO PP.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -972,6 +972,134 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SEO técnico</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Imagenes de producto sin optimizar (130-507 KB) afectaban tiempo de carga y Core Web Vitals (LCP), especialmente en mobile</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Corregido automatico - comprimidas con ImageMagick (quality 78, subsampling 4:2:0, metadata eliminada, resize maximo 1600px, mismo nombre de archivo). Ahorro total ~765 KB (36%) en bondiola, embutidos, mundialista, simple-ev, simple y tradicional.jpeg. odisea.jpeg sin cambios (ya estaba optimizada). Commit: https://github.com/lorenzoengraf10-dot/productosoatagonicos/commit/4d732d2</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mejora tiempo de carga y Core Web Vitals (LCP), especialmente en conexiones moviles</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SEO técnico</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>No fue posible auditar Core Web Vitals en vivo con Claude en Chrome (extension no conectada en esta sesion automatizada)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Auditoria realizada por lectura directa de HTML servido (Vercel y GitHub Pages) y del codigo fuente del repo</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Sin impacto en los hallazgos de hoy; recomendable correr una auditoria con Chrome en una sesion interactiva para medir LCP/CLS/INP reales</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Estacional</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Proximo partido de Argentina (cuartos de final vs Suiza, sabado 11/7 22:00 hs) sigue vigente: el partido aun no se jugo, sin cambios respecto de ayer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Sin accion - el dato ya esta reflejado correctamente en la tarjeta y el modal de Picada Mundialista</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Mantener el elemento estacional actualizado apenas se dispute el partido de esta noche (revisar rival/fecha del siguiente cruce o revertir el diseño si Argentina queda eliminada)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Conversión</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>El formulario de descuento (Formspree) exige completar 3 campos obligatorios (nombre, email, telefono) antes de mostrar el codigo de 10%, lo que agrega friccion frente a pedir un solo dato</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Propuesta pendiente de aprobacion - evaluar reducir a nombre + telefono (canal WhatsApp) o mostrar el codigo de inmediato y pedir el resto de los datos despues</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Propuesta pendiente</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Podria aumentar la tasa de registro al descuento del 10% y el pool de leads reutilizables para remarketing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
seo-log: registrar reduccion de formulario a email y cierre de definicion de dominio
</commit_message>
<xml_diff>
--- a/seo-log/vitacora de SEO PP.xlsx
+++ b/seo-log/vitacora de SEO PP.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1100,6 +1100,70 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Conversión</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Formulario de descuento pedia 3 campos (nombre, email, telefono), generando friccion</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Corregido automatico - aprobado por el dueno: se redujo el formulario a un solo campo (email). El telefono se obtiene por WhatsApp al reclamar el descuento. Commit: https://github.com/lorenzoengraf10-dot/productosoatagonicos/commit/b624e30</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Menos friccion en el registro, mas leads captados para remarketing por email</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SEO técnico</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Definicion pendiente sobre el dominio viejo de GitHub Pages (redirect o espejo)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Resuelto - el dueno confirmo que el dominio de GitHub Pages queda como espejo sin redirect, ya que usara Vercel como dominio principal de ahora en mas</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Cierra el bloqueo pendiente; no requiere mas seguimiento</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Bitacora Excel: franja resumen legible en celular (canal unico del dueno en el viaje) + directiva de actualizacion diaria
</commit_message>
<xml_diff>
--- a/seo-log/vitacora de SEO PP.xlsx
+++ b/seo-log/vitacora de SEO PP.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,10 +26,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00432820"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000b3d69"/>
+      <sz val="11"/>
     </font>
     <font>
       <i val="1"/>
@@ -37,22 +41,25 @@
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00F0E8D5"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCEAF6"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -91,20 +98,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -471,12 +481,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -489,271 +499,279 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Una fila por día: lo logrado y lo pendiente a futuro. Complementa bitacora.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+          <t>🔔 ÚLTIMA CORRIDA 17/07  ·  MODO VACACIONES ACTIVO (volvés el 2/8)  ·  ¿NECESITO ALGO DE VOS?: NO por ahora  ·  PRÓXIMO HITO: resultado de la final 19/07 (se resuelve solo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Una fila por día: lo logrado y lo pendiente a futuro. Se actualiza en cada corrida automática (8am). Complementa bitacora.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Día</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Logros del día</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Mejora del día</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Pendiente / A futuro</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Estado Mundial / Vacaciones</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="56" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Vie</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Revisión total de código (sin bugs). productos.json creado como fuente del catálogo; JSON-LD Product/Offer x7; WebP+fallback; SEO local (geo+keywords); sección Prueba social integrada.</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Migración del catálogo a productos.json + JSON-LD de productos</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Render dinámico de tarjetas desde JSON (pospuesto por conversión)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Revisión total de código (sin bugs). productos.json como fuente del catálogo; JSON-LD Product/Offer x7; WebP+fallback; SEO local; sección Prueba social integrada.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Migración del catálogo a productos.json + JSON-LD</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Render dinámico de tarjetas desde JSON (pospuesto)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Mundial en curso</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Sáb</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Lanzamiento Gran Promoción Mundialista; aura Argentina; varios fixes mobile (modal scroll, precio $, recorte fotos); form cableado a MailerLite; deploy prod corregido.</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Lanzamiento Gran Promoción Mundialista; aura Argentina; fixes mobile (modal scroll, precio $, fotos); form cableado a MailerLite; deploy corregido.</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Aura Mundial + tarjeta Mundialista nueva</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>simple.html con precios viejos (ignorar, decisión del dueño)</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Mundial — fase de grupos/eliminatorias</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Mundial — eliminatorias</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Dom</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Auditoría OK; width/height en imágenes (CLS); fuentes Google no bloqueantes; límite de pedidos Mundialista.</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>width/height en 9 &lt;img&gt; + fuentes async</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Activar bienvenida MailerLite (luego cerrado por el dueño)</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Medir LCP real en móvil</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Mundial en curso</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Lun</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Auditoría OK; AVIF en catálogo (−38% peso, Mundialista −50%); GitHub Pages sincronizado.</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>AVIF como primer &lt;source&gt; de cada &lt;picture&gt;</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Medir LCP real en móvil (&lt;2,5s)</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Mundial en curso</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Semifinal: Argentina 2-1 Inglaterra → FINAL. Tarjeta a Final vs España; catálogo reactivado (5/5 InStock); aviso pausa 16/07; preload imagen LCP; og/twitter image alt.</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>preload de la imagen LCP del hero + og/twitter image alt</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Semifinal: Argentina 2-1 Inglaterra → FINAL. Tarjeta a Final vs España; catálogo reactivado (5/5); aviso pausa 16/07; preload imagen LCP; og/twitter image alt.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>preload de imagen LCP + og/twitter image alt</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Reversión paleta post-Mundial (tras 19/07)</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Semifinal ganada → Final 19/07</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Semifinal ganada → Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Mié</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Auditoría OK; JSON-LD FoodEstablishment enriquecido (geo, areaServed, sameAs). Métricas GA4/IG/FB.</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>geo + areaServed + sameAs en FoodEstablishment</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>aggregateRating cuando haya reseñas</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Sin partido; Final 19/07 vs España</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="98" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Sin partido; Final 19/07</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="132" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Jue</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Auditoría OK (Vercel+Pages coherentes). Favicon + iconos de app + web app manifest (antes inexistentes). MODO VACACIONES activado (banner 2/8, pedidos repuntados a mail, cupón activo). Plan post-Mundial condicional pre-construido (MODO CAMPEÓN tras flag). Entregado docx de alta de Google Business Profile. Bitácora Excel reactivada.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Favicon + iconos de app + manifest PWA (branding/buscador móvil)</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Google Business Profile: alta+verificación (EN PAUSA hasta 2/8). Reapertura del sitio al volver (flag vacaciones off) + escribir a los mails juntados. Ejecutar plan campeón/reversión según resultado del 19/07.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Vacaciones hasta 2/8 · Final 19/07 (plan condicional armado)</t>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Auditoría OK. Favicon + iconos de app + manifest PWA (antes inexistentes). MODO VACACIONES activado (banner 2/8, pedidos → mail, cupón activo). MODO CAMPEÓN pre-construido (condicional al 19/07). Entregado docx alta Google Business. Bitácora Excel reactivada con resumen para celular.</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Favicon + iconos de app + manifest PWA</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Google Business: alta+verificación (EN PAUSA hasta 2/8). Reabrir el sitio al volver + escribir a los mails juntados. Plan campeón/reversión: se ejecuta solo el 20/07.</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Vacaciones hasta 2/8 · Final 19/07 (plan armado)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>